<commit_message>
Excel file for Aalborg with DK for 2 objectives
</commit_message>
<xml_diff>
--- a/AalborgResults/Two_Objectives/With PP conf and DK/Pareto-front with PP and DK.xlsx
+++ b/AalborgResults/Two_Objectives/With PP conf and DK/Pareto-front with PP and DK.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahbub\Documents\GitHub\EnergyPLANDomainKnowledgeEAStep1\AalborgResults\Two_Objectives\With PP conf and DK\from dendron\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahbub\Documents\GitHub\EnergyPLANDomainKnowledgeEAStep1\AalborgResults\Two_Objectives\With PP conf and DK\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -279,6 +279,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -288,8 +290,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2729,11 +2729,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="568607000"/>
-        <c:axId val="568606608"/>
+        <c:axId val="352844216"/>
+        <c:axId val="352845000"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="568607000"/>
+        <c:axId val="352844216"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.60000000000000009"/>
@@ -2839,13 +2839,13 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="568606608"/>
+        <c:crossAx val="352845000"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="568606608"/>
+        <c:axId val="352845000"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="6000"/>
@@ -2964,7 +2964,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="568607000"/>
+        <c:crossAx val="352844216"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="1000"/>
@@ -4554,11 +4554,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="568610920"/>
-        <c:axId val="568611312"/>
+        <c:axId val="352846568"/>
+        <c:axId val="352835200"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="568610920"/>
+        <c:axId val="352846568"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.60000000000000009"/>
@@ -4589,14 +4589,14 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="568611312"/>
+        <c:crossAx val="352835200"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
         <c:minorUnit val="0.1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="568611312"/>
+        <c:axId val="352835200"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4626,7 +4626,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="568610920"/>
+        <c:crossAx val="352846568"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4703,7 +4703,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>chp3</c:v>
+            <c:v>CHP</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
@@ -4714,7 +4714,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="3"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
@@ -6167,7 +6167,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>HP_C</c:v>
+            <c:v>HP</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="25400" cap="rnd">
@@ -6178,7 +6178,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="3"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
@@ -7635,11 +7635,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="568609744"/>
-        <c:axId val="568610136"/>
+        <c:axId val="352836376"/>
+        <c:axId val="352847352"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="568609744"/>
+        <c:axId val="352836376"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7659,6 +7659,62 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>CO2 Emission [Mt] </a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -7696,12 +7752,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="568610136"/>
+        <c:crossAx val="352847352"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="568610136"/>
+        <c:axId val="352847352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7721,6 +7777,62 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>Capacity [MW]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -7758,7 +7870,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="568609744"/>
+        <c:crossAx val="352836376"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7770,6 +7882,38 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -9327,45 +9471,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
       <c r="H1" s="3"/>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
       <c r="S1" s="3"/>
-      <c r="T1" s="8" t="s">
+      <c r="T1" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="U1" s="8"/>
-      <c r="W1" s="9" t="s">
+      <c r="U1" s="10"/>
+      <c r="W1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
-      <c r="AA1" s="9"/>
-      <c r="AB1" s="9"/>
-      <c r="AC1" s="9"/>
-      <c r="AD1" s="9"/>
-      <c r="AE1" s="9"/>
-      <c r="AF1" s="9"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -10121,7 +10265,7 @@
       <c r="R12">
         <v>1.28</v>
       </c>
-      <c r="S12" s="12"/>
+      <c r="S12" s="9"/>
       <c r="T12">
         <v>-0.55800000000000005</v>
       </c>
@@ -11277,7 +11421,7 @@
       <c r="R31">
         <v>1.23</v>
       </c>
-      <c r="S31" s="12"/>
+      <c r="S31" s="9"/>
       <c r="T31">
         <v>-0.53400000000000003</v>
       </c>
@@ -12128,7 +12272,7 @@
       <c r="R45">
         <v>1.17</v>
       </c>
-      <c r="S45" s="12"/>
+      <c r="S45" s="9"/>
       <c r="T45">
         <v>-0.50900000000000001</v>
       </c>
@@ -12674,7 +12818,7 @@
       <c r="R54">
         <v>1.1499999999999999</v>
       </c>
-      <c r="S54" s="12"/>
+      <c r="S54" s="9"/>
       <c r="T54">
         <v>-0.48699999999999999</v>
       </c>
@@ -12856,7 +13000,7 @@
       <c r="R57">
         <v>1.1200000000000001</v>
       </c>
-      <c r="S57" s="12"/>
+      <c r="S57" s="9"/>
       <c r="T57">
         <v>-0.48399999999999999</v>
       </c>
@@ -13221,7 +13365,7 @@
       <c r="R63">
         <v>1.1000000000000001</v>
       </c>
-      <c r="S63" s="12"/>
+      <c r="S63" s="9"/>
       <c r="T63">
         <v>-0.46500000000000002</v>
       </c>
@@ -13403,7 +13547,7 @@
       <c r="R66">
         <v>1.07</v>
       </c>
-      <c r="S66" s="12"/>
+      <c r="S66" s="9"/>
       <c r="T66">
         <v>-0.45500000000000002</v>
       </c>
@@ -13768,7 +13912,7 @@
       <c r="R72">
         <v>1.03</v>
       </c>
-      <c r="S72" s="12"/>
+      <c r="S72" s="9"/>
       <c r="T72">
         <v>-0.438</v>
       </c>
@@ -14070,7 +14214,7 @@
       <c r="R77">
         <v>1.02</v>
       </c>
-      <c r="S77" s="12"/>
+      <c r="S77" s="9"/>
       <c r="T77">
         <v>-0.42099999999999999</v>
       </c>
@@ -14191,7 +14335,7 @@
       <c r="R79">
         <v>0.98</v>
       </c>
-      <c r="S79" s="12"/>
+      <c r="S79" s="9"/>
       <c r="T79">
         <v>-0.41</v>
       </c>
@@ -14922,7 +15066,7 @@
       <c r="R91">
         <v>0.92</v>
       </c>
-      <c r="S91" s="12"/>
+      <c r="S91" s="9"/>
       <c r="T91">
         <v>-0.374</v>
       </c>
@@ -15043,7 +15187,7 @@
       <c r="R93">
         <v>0.91</v>
       </c>
-      <c r="S93" s="12"/>
+      <c r="S93" s="9"/>
       <c r="T93">
         <v>-0.36599999999999999</v>
       </c>
@@ -15833,7 +15977,7 @@
       <c r="R106">
         <v>0.79</v>
       </c>
-      <c r="S106" s="12"/>
+      <c r="S106" s="9"/>
       <c r="T106">
         <v>-0.27700000000000002</v>
       </c>
@@ -16137,7 +16281,7 @@
       <c r="R111">
         <v>0.75</v>
       </c>
-      <c r="S111" s="12"/>
+      <c r="S111" s="9"/>
       <c r="T111">
         <v>-0.249</v>
       </c>
@@ -16380,7 +16524,7 @@
       <c r="R115">
         <v>0.72</v>
       </c>
-      <c r="S115" s="12"/>
+      <c r="S115" s="9"/>
       <c r="T115">
         <v>-0.23499999999999999</v>
       </c>
@@ -17050,7 +17194,7 @@
       <c r="R126">
         <v>0.62</v>
       </c>
-      <c r="S126" s="12"/>
+      <c r="S126" s="9"/>
       <c r="T126">
         <v>-0.15</v>
       </c>
@@ -17598,7 +17742,7 @@
       <c r="R135">
         <v>0.52</v>
       </c>
-      <c r="S135" s="12"/>
+      <c r="S135" s="9"/>
       <c r="T135">
         <v>-7.4999999999999997E-2</v>
       </c>
@@ -17658,7 +17802,7 @@
       <c r="R136">
         <v>0.52</v>
       </c>
-      <c r="S136" s="12"/>
+      <c r="S136" s="9"/>
       <c r="T136">
         <v>-7.4999999999999997E-2</v>
       </c>
@@ -17779,7 +17923,7 @@
       <c r="R138">
         <v>0.55000000000000004</v>
       </c>
-      <c r="S138" s="12"/>
+      <c r="S138" s="9"/>
       <c r="T138">
         <v>-5.5E-2</v>
       </c>
@@ -18022,7 +18166,7 @@
       <c r="R142">
         <v>0.53</v>
       </c>
-      <c r="S142" s="12"/>
+      <c r="S142" s="9"/>
       <c r="T142">
         <v>-2.9000000000000001E-2</v>
       </c>
@@ -18997,7 +19141,7 @@
       <c r="R158">
         <v>0.36</v>
       </c>
-      <c r="S158" s="12"/>
+      <c r="S158" s="9"/>
       <c r="T158">
         <v>9.7000000000000003E-2</v>
       </c>
@@ -19057,7 +19201,7 @@
       <c r="R159">
         <v>0.36</v>
       </c>
-      <c r="S159" s="12"/>
+      <c r="S159" s="9"/>
       <c r="T159">
         <v>9.7000000000000003E-2</v>
       </c>
@@ -19298,7 +19442,7 @@
       <c r="R163">
         <v>0.31</v>
       </c>
-      <c r="S163" s="12"/>
+      <c r="S163" s="9"/>
       <c r="T163">
         <v>0.129</v>
       </c>
@@ -19480,7 +19624,7 @@
       <c r="R166">
         <v>0.28000000000000003</v>
       </c>
-      <c r="S166" s="12"/>
+      <c r="S166" s="9"/>
       <c r="T166">
         <v>0.14799999999999999</v>
       </c>
@@ -19784,7 +19928,7 @@
       <c r="R171">
         <v>0.21</v>
       </c>
-      <c r="S171" s="12"/>
+      <c r="S171" s="9"/>
       <c r="T171">
         <v>0.19700000000000001</v>
       </c>
@@ -19905,7 +20049,7 @@
       <c r="R173">
         <v>0.13</v>
       </c>
-      <c r="S173" s="12"/>
+      <c r="S173" s="9"/>
       <c r="T173">
         <v>0.20899999999999999</v>
       </c>
@@ -20270,7 +20414,7 @@
       <c r="R179">
         <v>0.11</v>
       </c>
-      <c r="S179" s="12"/>
+      <c r="S179" s="9"/>
       <c r="T179">
         <v>0.24199999999999999</v>
       </c>
@@ -21977,7 +22121,7 @@
       <c r="R207">
         <v>0</v>
       </c>
-      <c r="S207" s="12"/>
+      <c r="S207" s="9"/>
       <c r="T207">
         <v>0.433</v>
       </c>
@@ -22157,7 +22301,7 @@
       <c r="R210">
         <v>0</v>
       </c>
-      <c r="S210" s="12"/>
+      <c r="S210" s="9"/>
       <c r="T210">
         <v>0.44900000000000001</v>
       </c>
@@ -22217,7 +22361,7 @@
       <c r="R211">
         <v>0</v>
       </c>
-      <c r="S211" s="12"/>
+      <c r="S211" s="9"/>
       <c r="T211">
         <v>0.46100000000000002</v>
       </c>
@@ -22399,7 +22543,7 @@
       <c r="R214">
         <v>0</v>
       </c>
-      <c r="S214" s="12"/>
+      <c r="S214" s="9"/>
       <c r="T214">
         <v>0.48099999999999998</v>
       </c>
@@ -22520,7 +22664,7 @@
       <c r="R216">
         <v>0</v>
       </c>
-      <c r="S216" s="12"/>
+      <c r="S216" s="9"/>
       <c r="T216">
         <v>0.48899999999999999</v>
       </c>
@@ -22641,7 +22785,7 @@
       <c r="R218">
         <v>0</v>
       </c>
-      <c r="S218" s="12"/>
+      <c r="S218" s="9"/>
       <c r="T218">
         <v>0.503</v>
       </c>
@@ -22762,7 +22906,7 @@
       <c r="R220">
         <v>0</v>
       </c>
-      <c r="S220" s="12"/>
+      <c r="S220" s="9"/>
       <c r="T220">
         <v>0.52200000000000002</v>
       </c>
@@ -23930,20 +24074,20 @@
       </c>
     </row>
     <row r="240" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="S240" s="12"/>
+      <c r="S240" s="9"/>
     </row>
     <row r="241" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S241" s="12"/>
+      <c r="S241" s="9"/>
     </row>
     <row r="242" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S242" s="12"/>
-      <c r="T242" s="10" t="s">
+      <c r="S242" s="9"/>
+      <c r="T242" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="U242" s="10"/>
+      <c r="U242" s="12"/>
     </row>
     <row r="243" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S243" s="12"/>
+      <c r="S243" s="9"/>
       <c r="T243">
         <v>-0.56200000000000006</v>
       </c>
@@ -23952,7 +24096,7 @@
       </c>
     </row>
     <row r="244" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S244" s="12"/>
+      <c r="S244" s="9"/>
       <c r="T244">
         <v>0.61899999999999999</v>
       </c>
@@ -23961,7 +24105,7 @@
       </c>
     </row>
     <row r="245" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S245" s="12"/>
+      <c r="S245" s="9"/>
       <c r="T245">
         <v>0.61899999999999999</v>
       </c>
@@ -23970,7 +24114,7 @@
       </c>
     </row>
     <row r="246" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S246" s="12"/>
+      <c r="S246" s="9"/>
       <c r="T246">
         <v>0.36399999999999999</v>
       </c>
@@ -23979,7 +24123,7 @@
       </c>
     </row>
     <row r="247" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S247" s="12"/>
+      <c r="S247" s="9"/>
       <c r="T247">
         <v>0.42699999999999999</v>
       </c>
@@ -23988,7 +24132,7 @@
       </c>
     </row>
     <row r="248" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S248" s="12"/>
+      <c r="S248" s="9"/>
       <c r="T248">
         <v>-0.40899999999999997</v>
       </c>
@@ -23997,7 +24141,7 @@
       </c>
     </row>
     <row r="249" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S249" s="12"/>
+      <c r="S249" s="9"/>
       <c r="T249">
         <v>-0.56000000000000005</v>
       </c>
@@ -24006,7 +24150,7 @@
       </c>
     </row>
     <row r="250" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S250" s="12"/>
+      <c r="S250" s="9"/>
       <c r="T250">
         <v>-0.35599999999999998</v>
       </c>
@@ -24015,7 +24159,7 @@
       </c>
     </row>
     <row r="251" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S251" s="12"/>
+      <c r="S251" s="9"/>
       <c r="T251">
         <v>0.53500000000000003</v>
       </c>
@@ -24024,7 +24168,7 @@
       </c>
     </row>
     <row r="252" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S252" s="12"/>
+      <c r="S252" s="9"/>
       <c r="T252">
         <v>-0.42599999999999999</v>
       </c>
@@ -24033,7 +24177,7 @@
       </c>
     </row>
     <row r="253" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S253" s="12"/>
+      <c r="S253" s="9"/>
       <c r="T253">
         <v>-0.32800000000000001</v>
       </c>
@@ -24042,7 +24186,7 @@
       </c>
     </row>
     <row r="254" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S254" s="12"/>
+      <c r="S254" s="9"/>
       <c r="T254">
         <v>-0.54300000000000004</v>
       </c>
@@ -24051,7 +24195,7 @@
       </c>
     </row>
     <row r="255" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S255" s="12"/>
+      <c r="S255" s="9"/>
       <c r="T255">
         <v>-0.55800000000000005</v>
       </c>
@@ -24060,7 +24204,7 @@
       </c>
     </row>
     <row r="256" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S256" s="12"/>
+      <c r="S256" s="9"/>
       <c r="T256">
         <v>9.9000000000000005E-2</v>
       </c>
@@ -24069,7 +24213,7 @@
       </c>
     </row>
     <row r="257" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S257" s="12"/>
+      <c r="S257" s="9"/>
       <c r="T257">
         <v>0.48599999999999999</v>
       </c>
@@ -24078,7 +24222,7 @@
       </c>
     </row>
     <row r="258" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S258" s="12"/>
+      <c r="S258" s="9"/>
       <c r="T258">
         <v>0.24299999999999999</v>
       </c>
@@ -24087,7 +24231,7 @@
       </c>
     </row>
     <row r="259" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S259" s="12"/>
+      <c r="S259" s="9"/>
       <c r="T259">
         <v>-0.48199999999999998</v>
       </c>
@@ -24096,7 +24240,7 @@
       </c>
     </row>
     <row r="260" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S260" s="12"/>
+      <c r="S260" s="9"/>
       <c r="T260">
         <v>-0.56100000000000005</v>
       </c>
@@ -24105,7 +24249,7 @@
       </c>
     </row>
     <row r="261" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S261" s="12"/>
+      <c r="S261" s="9"/>
       <c r="T261">
         <v>-9.2999999999999999E-2</v>
       </c>
@@ -24114,7 +24258,7 @@
       </c>
     </row>
     <row r="262" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S262" s="12"/>
+      <c r="S262" s="9"/>
       <c r="T262">
         <v>-0.13</v>
       </c>
@@ -24123,7 +24267,7 @@
       </c>
     </row>
     <row r="263" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S263" s="12"/>
+      <c r="S263" s="9"/>
       <c r="T263">
         <v>6.5000000000000002E-2</v>
       </c>
@@ -24132,7 +24276,7 @@
       </c>
     </row>
     <row r="264" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S264" s="12"/>
+      <c r="S264" s="9"/>
       <c r="T264">
         <v>-0.182</v>
       </c>
@@ -24141,7 +24285,7 @@
       </c>
     </row>
     <row r="265" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S265" s="12"/>
+      <c r="S265" s="9"/>
       <c r="T265">
         <v>-0.55300000000000005</v>
       </c>
@@ -24150,7 +24294,7 @@
       </c>
     </row>
     <row r="266" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S266" s="12"/>
+      <c r="S266" s="9"/>
       <c r="T266">
         <v>1E-3</v>
       </c>
@@ -24159,7 +24303,7 @@
       </c>
     </row>
     <row r="267" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S267" s="12"/>
+      <c r="S267" s="9"/>
       <c r="T267">
         <v>0.30099999999999999</v>
       </c>
@@ -24168,7 +24312,7 @@
       </c>
     </row>
     <row r="268" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S268" s="12"/>
+      <c r="S268" s="9"/>
       <c r="T268">
         <v>-0.10199999999999999</v>
       </c>
@@ -24177,7 +24321,7 @@
       </c>
     </row>
     <row r="269" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S269" s="12"/>
+      <c r="S269" s="9"/>
       <c r="T269">
         <v>-0.20699999999999999</v>
       </c>
@@ -24186,7 +24330,7 @@
       </c>
     </row>
     <row r="270" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S270" s="12"/>
+      <c r="S270" s="9"/>
       <c r="T270">
         <v>-0.55400000000000005</v>
       </c>
@@ -24195,7 +24339,7 @@
       </c>
     </row>
     <row r="271" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S271" s="12"/>
+      <c r="S271" s="9"/>
       <c r="T271">
         <v>-0.47199999999999998</v>
       </c>
@@ -24204,7 +24348,7 @@
       </c>
     </row>
     <row r="272" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S272" s="12"/>
+      <c r="S272" s="9"/>
       <c r="T272">
         <v>-0.441</v>
       </c>
@@ -24213,7 +24357,7 @@
       </c>
     </row>
     <row r="273" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S273" s="12"/>
+      <c r="S273" s="9"/>
       <c r="T273">
         <v>-0.51600000000000001</v>
       </c>
@@ -24222,7 +24366,7 @@
       </c>
     </row>
     <row r="274" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S274" s="12"/>
+      <c r="S274" s="9"/>
       <c r="T274">
         <v>-0.55100000000000005</v>
       </c>
@@ -24231,7 +24375,7 @@
       </c>
     </row>
     <row r="275" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S275" s="12"/>
+      <c r="S275" s="9"/>
       <c r="T275">
         <v>-0.49299999999999999</v>
       </c>
@@ -24240,7 +24384,7 @@
       </c>
     </row>
     <row r="276" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S276" s="12"/>
+      <c r="S276" s="9"/>
       <c r="T276">
         <v>-0.55700000000000005</v>
       </c>
@@ -24249,7 +24393,7 @@
       </c>
     </row>
     <row r="277" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S277" s="12"/>
+      <c r="S277" s="9"/>
       <c r="T277">
         <v>-0.54</v>
       </c>
@@ -24258,7 +24402,7 @@
       </c>
     </row>
     <row r="278" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S278" s="12"/>
+      <c r="S278" s="9"/>
       <c r="T278">
         <v>-0.437</v>
       </c>
@@ -24267,7 +24411,7 @@
       </c>
     </row>
     <row r="279" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S279" s="12"/>
+      <c r="S279" s="9"/>
       <c r="T279">
         <v>-0.53400000000000003</v>
       </c>
@@ -24276,7 +24420,7 @@
       </c>
     </row>
     <row r="280" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S280" s="12"/>
+      <c r="S280" s="9"/>
       <c r="T280">
         <v>-0.504</v>
       </c>
@@ -24285,7 +24429,7 @@
       </c>
     </row>
     <row r="281" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S281" s="12"/>
+      <c r="S281" s="9"/>
       <c r="T281">
         <v>-3.1E-2</v>
       </c>
@@ -24294,7 +24438,7 @@
       </c>
     </row>
     <row r="282" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S282" s="12"/>
+      <c r="S282" s="9"/>
       <c r="T282">
         <v>0.44900000000000001</v>
       </c>
@@ -24303,7 +24447,7 @@
       </c>
     </row>
     <row r="283" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S283" s="12"/>
+      <c r="S283" s="9"/>
       <c r="T283">
         <v>0.03</v>
       </c>
@@ -24312,7 +24456,7 @@
       </c>
     </row>
     <row r="284" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S284" s="12"/>
+      <c r="S284" s="9"/>
       <c r="T284">
         <v>0.19</v>
       </c>
@@ -24321,7 +24465,7 @@
       </c>
     </row>
     <row r="285" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S285" s="12"/>
+      <c r="S285" s="9"/>
       <c r="T285">
         <v>-0.23799999999999999</v>
       </c>
@@ -24330,7 +24474,7 @@
       </c>
     </row>
     <row r="286" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S286" s="12"/>
+      <c r="S286" s="9"/>
       <c r="T286">
         <v>-0.52600000000000002</v>
       </c>
@@ -24339,7 +24483,7 @@
       </c>
     </row>
     <row r="287" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S287" s="12"/>
+      <c r="S287" s="9"/>
       <c r="T287">
         <v>-0.48599999999999999</v>
       </c>
@@ -24348,7 +24492,7 @@
       </c>
     </row>
     <row r="288" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S288" s="12"/>
+      <c r="S288" s="9"/>
       <c r="T288">
         <v>-0.20499999999999999</v>
       </c>
@@ -24357,7 +24501,7 @@
       </c>
     </row>
     <row r="289" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S289" s="12"/>
+      <c r="S289" s="9"/>
       <c r="T289">
         <v>-0.52900000000000003</v>
       </c>
@@ -24366,7 +24510,7 @@
       </c>
     </row>
     <row r="290" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S290" s="12"/>
+      <c r="S290" s="9"/>
       <c r="T290">
         <v>0.215</v>
       </c>
@@ -24375,7 +24519,7 @@
       </c>
     </row>
     <row r="291" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S291" s="12"/>
+      <c r="S291" s="9"/>
       <c r="T291">
         <v>-0.35899999999999999</v>
       </c>
@@ -24384,7 +24528,7 @@
       </c>
     </row>
     <row r="292" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S292" s="12"/>
+      <c r="S292" s="9"/>
       <c r="T292">
         <v>-0.501</v>
       </c>
@@ -24393,7 +24537,7 @@
       </c>
     </row>
     <row r="293" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S293" s="12"/>
+      <c r="S293" s="9"/>
       <c r="T293">
         <v>-0.53200000000000003</v>
       </c>
@@ -24402,7 +24546,7 @@
       </c>
     </row>
     <row r="294" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S294" s="12"/>
+      <c r="S294" s="9"/>
       <c r="T294">
         <v>-0.27200000000000002</v>
       </c>
@@ -24411,7 +24555,7 @@
       </c>
     </row>
     <row r="295" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S295" s="12"/>
+      <c r="S295" s="9"/>
       <c r="T295">
         <v>0.26300000000000001</v>
       </c>
@@ -24420,7 +24564,7 @@
       </c>
     </row>
     <row r="296" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S296" s="12"/>
+      <c r="S296" s="9"/>
       <c r="T296">
         <v>-0.14599999999999999</v>
       </c>
@@ -24429,7 +24573,7 @@
       </c>
     </row>
     <row r="297" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S297" s="12"/>
+      <c r="S297" s="9"/>
       <c r="T297">
         <v>-0.49199999999999999</v>
       </c>
@@ -24438,7 +24582,7 @@
       </c>
     </row>
     <row r="298" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S298" s="12"/>
+      <c r="S298" s="9"/>
       <c r="T298">
         <v>0.60299999999999998</v>
       </c>
@@ -24447,7 +24591,7 @@
       </c>
     </row>
     <row r="299" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S299" s="12"/>
+      <c r="S299" s="9"/>
       <c r="T299">
         <v>-0.53500000000000003</v>
       </c>
@@ -24456,7 +24600,7 @@
       </c>
     </row>
     <row r="300" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S300" s="12"/>
+      <c r="S300" s="9"/>
       <c r="T300">
         <v>-0.54600000000000004</v>
       </c>
@@ -24465,7 +24609,7 @@
       </c>
     </row>
     <row r="301" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S301" s="12"/>
+      <c r="S301" s="9"/>
       <c r="T301">
         <v>-0.54800000000000004</v>
       </c>
@@ -24474,7 +24618,7 @@
       </c>
     </row>
     <row r="302" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S302" s="12"/>
+      <c r="S302" s="9"/>
       <c r="T302">
         <v>0.56799999999999995</v>
       </c>
@@ -24483,7 +24627,7 @@
       </c>
     </row>
     <row r="303" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S303" s="12"/>
+      <c r="S303" s="9"/>
       <c r="T303">
         <v>-0.55000000000000004</v>
       </c>
@@ -24492,7 +24636,7 @@
       </c>
     </row>
     <row r="304" spans="19:21" x14ac:dyDescent="0.25">
-      <c r="S304" s="12"/>
+      <c r="S304" s="9"/>
       <c r="T304">
         <v>0.35</v>
       </c>
@@ -24501,29 +24645,29 @@
       </c>
     </row>
     <row r="305" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A305" s="11"/>
-      <c r="B305" s="11"/>
-      <c r="C305" s="11"/>
-      <c r="D305" s="11"/>
-      <c r="E305" s="11"/>
-      <c r="F305" s="11"/>
-      <c r="G305" s="11"/>
-      <c r="H305" s="11"/>
-      <c r="I305" s="11"/>
-      <c r="J305" s="11"/>
-      <c r="K305" s="11"/>
-      <c r="L305" s="11"/>
-      <c r="M305" s="11"/>
-      <c r="N305" s="11"/>
-      <c r="O305" s="11"/>
-      <c r="P305" s="11"/>
-      <c r="Q305" s="11"/>
-      <c r="R305" s="11"/>
-      <c r="S305" s="11"/>
-      <c r="T305" s="11">
+      <c r="A305" s="8"/>
+      <c r="B305" s="8"/>
+      <c r="C305" s="8"/>
+      <c r="D305" s="8"/>
+      <c r="E305" s="8"/>
+      <c r="F305" s="8"/>
+      <c r="G305" s="8"/>
+      <c r="H305" s="8"/>
+      <c r="I305" s="8"/>
+      <c r="J305" s="8"/>
+      <c r="K305" s="8"/>
+      <c r="L305" s="8"/>
+      <c r="M305" s="8"/>
+      <c r="N305" s="8"/>
+      <c r="O305" s="8"/>
+      <c r="P305" s="8"/>
+      <c r="Q305" s="8"/>
+      <c r="R305" s="8"/>
+      <c r="S305" s="8"/>
+      <c r="T305" s="8">
         <v>-0.51100000000000001</v>
       </c>
-      <c r="U305" s="11">
+      <c r="U305" s="8">
         <v>4430</v>
       </c>
     </row>
@@ -24551,7 +24695,7 @@
         <v>3153</v>
       </c>
     </row>
-    <row r="309" spans="1:21" s="11" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:21" s="8" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A309"/>
       <c r="B309"/>
       <c r="C309"/>
@@ -24854,10 +24998,10 @@
     <mergeCell ref="T242:U242"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:A239">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="2" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>83</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38083,72 +38227,72 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A230:U230">
-    <cfRule type="cellIs" dxfId="15" priority="14" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A230">
-    <cfRule type="cellIs" dxfId="14" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="13" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A231:U231">
-    <cfRule type="cellIs" dxfId="13" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A231">
-    <cfRule type="cellIs" dxfId="12" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="11" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A232:U233">
-    <cfRule type="cellIs" dxfId="11" priority="10" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="10" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A232:A233">
-    <cfRule type="cellIs" dxfId="10" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A234:U234">
-    <cfRule type="cellIs" dxfId="9" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A234">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A235:U235">
-    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A235">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A236:U236">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A236">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A237:U237">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A237">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Aalborg result files are updated
</commit_message>
<xml_diff>
--- a/AalborgResults/Two_Objectives/With PP conf and DK/Pareto-front with PP and DK.xlsx
+++ b/AalborgResults/Two_Objectives/With PP conf and DK/Pareto-front with PP and DK.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="57">
   <si>
     <t>CHP3</t>
   </si>
@@ -294,7 +294,27 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2729,11 +2749,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="352844216"/>
-        <c:axId val="352845000"/>
+        <c:axId val="323662656"/>
+        <c:axId val="323663832"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="352844216"/>
+        <c:axId val="323662656"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.60000000000000009"/>
@@ -2839,13 +2859,13 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="352845000"/>
+        <c:crossAx val="323663832"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="352845000"/>
+        <c:axId val="323663832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="6000"/>
@@ -2964,7 +2984,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="352844216"/>
+        <c:crossAx val="323662656"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="1000"/>
@@ -4554,11 +4574,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="352846568"/>
-        <c:axId val="352835200"/>
+        <c:axId val="323653248"/>
+        <c:axId val="323665792"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="352846568"/>
+        <c:axId val="323653248"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.60000000000000009"/>
@@ -4589,14 +4609,14 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="352835200"/>
+        <c:crossAx val="323665792"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
         <c:minorUnit val="0.1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="352835200"/>
+        <c:axId val="323665792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4626,7 +4646,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="352846568"/>
+        <c:crossAx val="323653248"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7635,11 +7655,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="352836376"/>
-        <c:axId val="352847352"/>
+        <c:axId val="323666576"/>
+        <c:axId val="323667752"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="352836376"/>
+        <c:axId val="323666576"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7752,12 +7772,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="352847352"/>
+        <c:crossAx val="323667752"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="352847352"/>
+        <c:axId val="323667752"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7870,7 +7890,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="352836376"/>
+        <c:crossAx val="323666576"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -24998,11 +25018,11 @@
     <mergeCell ref="T242:U242"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:A239">
-    <cfRule type="cellIs" dxfId="15" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+      <formula>83</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="greaterThan">
       <formula>$C$4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
-      <formula>83</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -38227,72 +38247,72 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A230:U230">
-    <cfRule type="cellIs" dxfId="13" priority="14" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="14" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A230">
-    <cfRule type="cellIs" dxfId="12" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="13" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A231:U231">
-    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="12" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A231">
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="11" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A232:U233">
-    <cfRule type="cellIs" dxfId="9" priority="10" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="10" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A232:A233">
-    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="9" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A234:U234">
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="8" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A234">
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A235:U235">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A235">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A236:U236">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A236">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="greaterThan">
       <formula>$C$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A237:U237">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A237">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38302,133 +38322,236 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:V22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>37</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>38</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>0.03</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>20</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>0.03</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>32</v>
       </c>
-      <c r="B5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="B6">
         <v>1500</v>
       </c>
-      <c r="B6">
-        <v>4160</v>
-      </c>
-      <c r="C6">
-        <f>(A6*$B$2)*$C$2/(1-(1+$C$2)^(-$D$2))</f>
+      <c r="D6">
+        <f>(B6*$C$2)*$D$2/(1-(1+$D$2)^(-$E$2))</f>
         <v>100.82356139528873</v>
       </c>
-      <c r="D6">
-        <f>A6*$B$2*$E$2</f>
+      <c r="E6">
+        <f>B6*$C$2*$F$2</f>
         <v>45</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>0.19</v>
       </c>
-      <c r="F6">
-        <f>E6*10^6</f>
+      <c r="G6">
+        <f>F6*10^6</f>
         <v>190000</v>
       </c>
-      <c r="G6">
-        <f>F6*$F$2</f>
+      <c r="H6">
+        <f>G6*$G$2</f>
         <v>190000</v>
       </c>
-      <c r="H6">
-        <f>G6/10^6</f>
+      <c r="I6">
+        <f>H6/10^6</f>
         <v>0.19</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>194</v>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
       </c>
       <c r="B7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <f>(B7*$C$2)*$D$2/(1-(1+$D$2)^(-$E$2))</f>
+        <v>67.215707596859161</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>4739</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>196</v>
+      </c>
+      <c r="C11">
         <v>4033</v>
       </c>
-      <c r="C7">
-        <f>(A7*$B$2)*$C$2/(1-(1+$C$2)^(-$D$2))</f>
-        <v>13.039847273790675</v>
-      </c>
-      <c r="D7">
-        <f>A7*$B$2*$E$2</f>
-        <v>5.8199999999999994</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C10">
-        <f>B6-D10</f>
-        <v>4033.036285878502</v>
-      </c>
-      <c r="D10">
-        <f>C6+D6-C7-D7</f>
-        <v>126.96371412149804</v>
+      <c r="D11">
+        <f>(B11*$C$2)*$D$2/(1-(1+$D$2)^(-$E$2))</f>
+        <v>13.174278688984396</v>
+      </c>
+      <c r="E11">
+        <f>B11*$C$2*$F$2</f>
+        <v>5.88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <f>C8-E14</f>
+        <v>4612.2307172936953</v>
+      </c>
+      <c r="E14">
+        <f>D6+E6-D11-E11</f>
+        <v>126.76928270630432</v>
+      </c>
+    </row>
+    <row r="22" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>54</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>84</v>
+      </c>
+      <c r="E22">
+        <v>1449</v>
+      </c>
+      <c r="F22">
+        <v>540</v>
+      </c>
+      <c r="G22">
+        <v>243</v>
+      </c>
+      <c r="H22">
+        <v>196</v>
+      </c>
+      <c r="I22" s="7"/>
+      <c r="J22">
+        <v>0.01</v>
+      </c>
+      <c r="K22">
+        <v>0.02</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22">
+        <v>1.08</v>
+      </c>
+      <c r="O22">
+        <v>1.73</v>
+      </c>
+      <c r="P22">
+        <v>0.05</v>
+      </c>
+      <c r="Q22">
+        <v>0.13</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>1.22</v>
+      </c>
+      <c r="T22" s="7"/>
+      <c r="U22">
+        <v>-0.53100000000000003</v>
+      </c>
+      <c r="V22">
+        <v>4649</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B22">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+      <formula>83</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" operator="greaterThan" id="{20216D99-A9EF-44A9-8C47-157535823EAD}">
+            <xm:f>Sheet2!$C$4</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>B22</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 

</xml_diff>